<commit_message>
ci: add GitHub Actions for tests and performance
- tests.yml: typecheck, prettier and k6 script checks, k6 smoke (PF001) and
  Playwright on api/chromium/firefox/webkit on every push and pull request
- perf.yml: load and Web Vitals scripts nightly and on demand, one at a time
- PF005-PF007 rewritten to match the performance test case sheet
- format the code with prettier so the format check passes
</commit_message>
<xml_diff>
--- a/test-cases/Demoblaze_TestCases_Performance.xlsx
+++ b/test-cases/Demoblaze_TestCases_Performance.xlsx
@@ -1,89 +1,87 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <workbookPr date1904="0"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1" showHorizontalScroll="1" showVerticalScroll="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="Performance" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Performance" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Performance!$A$1:$P$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Performance!$A$1:$P$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Performance!$A$1:$P$8</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
-    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="124">
   <si>
     <t xml:space="preserve">Demoblaze – Performance Test Cases (Login &amp; Cart)</t>
   </si>
   <si>
-    <t xml:space="preserve">Application</t>
+    <t>Application</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.demoblaze.com/ (API: https://api.demoblaze.com)</t>
   </si>
   <si>
-    <t xml:space="preserve">Scope</t>
+    <t>Scope</t>
   </si>
   <si>
     <t xml:space="preserve">Login, Cart – API latency under load + frontend Web Vitals</t>
   </si>
   <si>
-    <t xml:space="preserve">Tool</t>
+    <t>Tool</t>
   </si>
   <si>
     <t xml:space="preserve">k6 (HTTP + k6/browser)</t>
   </si>
   <si>
-    <t xml:space="preserve">Author</t>
+    <t>Author</t>
   </si>
   <si>
     <t xml:space="preserve">Nolan Tran</t>
   </si>
   <si>
-    <t xml:space="preserve">Version</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Created</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-28</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coverage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Login</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cart</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smoke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Load</t>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>1.0</t>
+  </si>
+  <si>
+    <t>Created</t>
+  </si>
+  <si>
+    <t>2026-10-28</t>
+  </si>
+  <si>
+    <t>Coverage</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Cart</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Smoke</t>
+  </si>
+  <si>
+    <t>Load</t>
   </si>
   <si>
     <t xml:space="preserve">Web Vitals</t>
@@ -92,13 +90,13 @@
     <t xml:space="preserve">Execution status</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fail</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blocked</t>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Fail</t>
+  </si>
+  <si>
+    <t>Blocked</t>
   </si>
   <si>
     <t xml:space="preserve">Not Run</t>
@@ -110,19 +108,19 @@
     <t xml:space="preserve">Load profiles</t>
   </si>
   <si>
-    <t xml:space="preserve">Profile</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Purpose</t>
+    <t>Profile</t>
+  </si>
+  <si>
+    <t>Shape</t>
+  </si>
+  <si>
+    <t>Purpose</t>
   </si>
   <si>
     <t xml:space="preserve">When it runs</t>
   </si>
   <si>
-    <t xml:space="preserve">smoke</t>
+    <t>smoke</t>
   </si>
   <si>
     <t xml:space="preserve">1 VU, 1 min</t>
@@ -134,7 +132,7 @@
     <t xml:space="preserve">Every push / MR</t>
   </si>
   <si>
-    <t xml:space="preserve">load</t>
+    <t>load</t>
   </si>
   <si>
     <t xml:space="preserve">0→10 VUs (1 min), 10 VUs (3 min), 10→0 (1 min)</t>
@@ -146,7 +144,7 @@
     <t xml:space="preserve">Nightly / manual</t>
   </si>
   <si>
-    <t xml:space="preserve">browser</t>
+    <t>browser</t>
   </si>
   <si>
     <t xml:space="preserve">1 VU, 5 iterations, Chromium</t>
@@ -158,19 +156,19 @@
     <t xml:space="preserve">TC ID</t>
   </si>
   <si>
-    <t xml:space="preserve">Feature</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Title</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Priority</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Target</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preconditions</t>
+    <t>Feature</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Priority</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>Preconditions</t>
   </si>
   <si>
     <t xml:space="preserve">Load Profile</t>
@@ -179,34 +177,34 @@
     <t xml:space="preserve">Test Flow</t>
   </si>
   <si>
-    <t xml:space="preserve">Metrics</t>
+    <t>Metrics</t>
   </si>
   <si>
     <t xml:space="preserve">Threshold (Pass criteria)</t>
   </si>
   <si>
-    <t xml:space="preserve">Automation</t>
+    <t>Automation</t>
   </si>
   <si>
     <t xml:space="preserve">k6 Script</t>
   </si>
   <si>
-    <t xml:space="preserve">Status</t>
+    <t>Status</t>
   </si>
   <si>
     <t xml:space="preserve">Actual Result</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PF-001</t>
+    <t>Notes</t>
+  </si>
+  <si>
+    <t>PF-001</t>
   </si>
   <si>
     <t xml:space="preserve">Login API – smoke baseline</t>
   </si>
   <si>
-    <t xml:space="preserve">High</t>
+    <t>High</t>
   </si>
   <si>
     <t xml:space="preserve">POST https://api.demoblaze.com/login</t>
@@ -233,13 +231,13 @@
 checks rate &gt; 99%</t>
   </si>
   <si>
-    <t xml:space="preserve">k6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tests/performance/scenarios/login.k6.ts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pass</t>
+    <t>k6</t>
+  </si>
+  <si>
+    <t>tests/performance/scenarios/login.k6.ts</t>
+  </si>
+  <si>
+    <t>pass</t>
   </si>
   <si>
     <t xml:space="preserve">    checks
@@ -273,7 +271,7 @@
     <t xml:space="preserve">Runs on every push / MR</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-002</t>
+    <t>PF-002</t>
   </si>
   <si>
     <t xml:space="preserve">Login API – load</t>
@@ -315,7 +313,7 @@
     <t xml:space="preserve">Nightly / manual trigger</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-003</t>
+    <t>PF-003</t>
   </si>
   <si>
     <t xml:space="preserve">Add to cart API – load</t>
@@ -337,19 +335,40 @@
 checks</t>
   </si>
   <si>
-    <t xml:space="preserve">tests/performance/scenarios/cart.k6.ts</t>
+    <t>tests/performance/scenarios/cart.k6.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TOTAL RESULTS 
+    checks_total.......: 1682    4.647349/s
+    checks_succeeded...: 100.00% 1682 out of 1682
+    checks_failed......: 0.00%   0 out of 1682
+    ✓ add to cart status 200
+    HTTP
+    http_req_duration..............: avg=484.02ms min=253.22ms med=277.2ms  max=11.25s p(90)=898.39ms p(95)=1.73s
+      { expected_response:true }...: avg=484.02ms min=253.22ms med=277.2ms  max=11.25s p(90)=898.39ms p(95)=1.73s
+      { name:addtocart }...........: avg=450.61ms min=253.22ms med=277.11ms max=6.28s  p(90)=841.51ms p(95)=1.66s
+    http_req_failed................: 0.00%  0 out of 1689
+    http_reqs......................: 1689   4.66669/s
+    EXECUTION
+    iteration_duration.............: avg=1.45s    min=1.25s    med=1.27s    max=7.28s  p(90)=1.84s    p(95)=2.66s
+    iterations.....................: 1682   4.647349/s
+    vus............................: 0      min=0         max=10
+    vus_max........................: 10     min=10        max=10
+    NETWORK
+    data_received..................: 245 kB 677 B/s
+    data_sent......................: 418 kB 1.2 kB/s</t>
   </si>
   <si>
     <t xml:space="preserve">teardown() deletes created rows</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-004</t>
+    <t>PF-004</t>
   </si>
   <si>
     <t xml:space="preserve">View cart API – load with 5 items</t>
   </si>
   <si>
-    <t xml:space="preserve">Medium</t>
+    <t>Medium</t>
   </si>
   <si>
     <t xml:space="preserve">POST https://api.demoblaze.com/viewcart</t>
@@ -368,7 +387,31 @@
 checks</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-005</t>
+    <t xml:space="preserve">OTAL RESULTS 
+    checks_total.......: 4509    14.366251/s
+    checks_succeeded...: 100.00% 4509 out of 4509
+    checks_failed......: 0.00%   0 out of 4509
+    ✓ view cart status 200
+    ✓ cart has 5 lines
+    ✓ cart has the seeded products
+    HTTP
+    http_req_duration..............: avg=603.03ms min=252.11ms med=297.19ms max=3.83s  p(90)=1.61s p(95)=2.01s
+      { expected_response:true }...: avg=603.03ms min=252.11ms med=297.19ms max=3.83s  p(90)=1.61s p(95)=2.01s
+      { name:viewcart }............: avg=547.29ms min=252.11ms med=291.08ms max=3.83s  p(90)=1.42s p(95)=1.93s
+    http_req_failed................: 0.00%  0 out of 1564
+      { name:viewcart }............: 0.00%  0 out of 1503
+    http_reqs......................: 1564   4.983104/s
+    EXECUTION
+    iteration_duration.............: avg=1.62s    min=1.25s    med=1.29s    max=18.25s p(90)=2.43s p(95)=2.95s
+    iterations.....................: 1503   4.78875/s
+    vus............................: 0      min=0         max=10
+    vus_max........................: 10     min=10        max=10
+    NETWORK
+    data_received..................: 1.2 MB 4.0 kB/s
+    data_sent......................: 311 kB 992 B/s</t>
+  </si>
+  <si>
+    <t>PF-005</t>
   </si>
   <si>
     <t xml:space="preserve">Cart journey API – add → view → delete</t>
@@ -396,19 +439,57 @@
 checks rate &gt; 99%</t>
   </si>
   <si>
+    <t xml:space="preserve">    checks
+    ✓ 'rate&gt;0.99' rate=100.00%
+    http_req_duration{name:addtocart}
+    ✓ 'p(95)&lt;1800' p(95)=996.94ms
+    http_req_duration{name:deleteitem}
+    ✓ 'p(95)&lt;1800' p(95)=800.62ms
+    http_req_duration{name:viewcart}
+    ✓ 'p(95)&lt;1800' p(95)=753.69ms
+    http_req_failed
+    ✓ 'rate&lt;0.01' rate=0.00%
+    iteration_duration
+    ✓ 'p(95)&lt;6000' p(95)=5.15s
+  █ TOTAL RESULTS 
+    checks_total.......: 4064    13.283968/s
+    checks_succeeded...: 100.00% 4064 out of 4064
+    checks_failed......: 0.00%   0 out of 4064
+    ✓ add to cart status 200
+    ✓ cart has the added item
+    ✓ delete item status 200
+    ✓ deleted item is gone
+    HTTP
+    http_req_duration..............: avg=353.02ms min=237.8ms  med=274.39ms max=2.15s p(90)=341.18ms p(95)=804.34ms
+      { expected_response:true }...: avg=353.02ms min=237.8ms  med=274.39ms max=2.15s p(90)=341.18ms p(95)=804.34ms
+      { name:addtocart }...........: avg=360.5ms  min=252ms    med=273.79ms max=2.04s p(90)=345.63ms p(95)=996.94ms
+      { name:deleteitem }..........: avg=366.41ms min=260.57ms med=289.56ms max=2.15s p(90)=363.06ms p(95)=800.62ms
+      { name:viewcart }............: avg=342.01ms min=237.8ms  med=262.16ms max=2.15s p(90)=329.76ms p(95)=753.69ms
+    http_req_failed................: 0.00%  0 out of 4075
+    http_reqs......................: 4075   13.319924/s
+    EXECUTION
+    iteration_duration.............: avg=2.41s    min=2.01s    med=2.11s    max=9.01s p(90)=2.28s    p(95)=5.15s   
+    iterations.....................: 1016   3.320992/s
+    vus............................: 0      min=0         max=10
+    vus_max........................: 10     min=10        max=10
+    NETWORK
+    data_received..................: 910 kB 3.0 kB/s
+    data_sent......................: 783 kB 2.6 kB/s</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cart stays empty after each iteration</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-006</t>
+    <t>PF-006</t>
   </si>
   <si>
     <t xml:space="preserve">Home page (login entry) – Web Vitals</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.demoblaze.com/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">None</t>
+    <t>https://www.demoblaze.com/</t>
+  </si>
+  <si>
+    <t>None</t>
   </si>
   <si>
     <t xml:space="preserve">browser: 1 VU, 5 iterations (Chromium)</t>
@@ -428,19 +509,56 @@
 TTFB p(75) &lt; 800 ms</t>
   </si>
   <si>
-    <t xml:space="preserve">tests/performance/scenarios/web-vitals.k6.ts</t>
+    <t>tests/performance/scenarios/web-vitals.k6.ts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THRESHOLDS 
+    browser_web_vital_cls
+    ✓ 'p(75)&lt;0.1' p(75)=0.079326
+    browser_web_vital_fcp
+    ✓ 'p(75)&lt;1800' p(75)=664ms
+    browser_web_vital_lcp
+    ✓ 'p(75)&lt;2500' p(75)=664ms
+    browser_web_vital_ttfb
+    ✓ 'p(75)&lt;800' p(75)=350.59ms
+    checks
+    ✓ 'rate&gt;0.99' rate=100.00%
+  █ TOTAL RESULTS 
+    checks_total.......: 5       0.390492/s
+    checks_succeeded...: 100.00% 5 out of 5
+    checks_failed......: 0.00%   0 out of 5
+    ✓ Log in modal opens
+    EXECUTION
+    iteration_duration..........: avg=2.35s    min=1.75s    med=2.13s    max=3.73s    p(90)=3.14s    p(95)=3.43s   
+    iterations..................: 5     0.390492/s
+    vus.........................: 1     min=1        max=1
+    vus_max.....................: 1     min=1        max=1
+    NETWORK
+    data_received...............: 0 B   0 B/s
+    data_sent...................: 0 B   0 B/s
+    BROWSER
+    browser_data_received.......: 15 MB 1.2 MB/s
+    browser_data_sent...........: 79 kB 6.2 kB/s
+    browser_http_req_duration...: avg=239.65ms min=29.25ms  med=258.15ms max=2.25s    p(90)=352.31ms p(95)=383.8ms 
+    browser_http_req_failed.....: 0.00% 0 out of 155
+    WEB_VITALS
+    browser_web_vital_cls.......: avg=0.075353 min=0.063025 med=0.065209 max=0.106008 p(90)=0.095335 p(95)=0.100671
+    browser_web_vital_fcp.......: avg=688.8ms  min=628ms    med=660ms    max=852ms    p(90)=776.8ms  p(95)=814.4ms 
+    browser_web_vital_inp.......: avg=17.6ms   min=16ms     med=16ms     max=24ms     p(90)=20.8ms   p(95)=22.4ms  
+    browser_web_vital_lcp.......: avg=688.8ms  min=628ms    med=660ms    max=852ms    p(90)=776.8ms  p(95)=814.4ms 
+    browser_web_vital_ttfb......: avg=360.8ms  min=326.29ms med=340.1ms  max=449.09ms p(90)=409.69ms p(95)=429.39ms</t>
   </si>
   <si>
     <t xml:space="preserve">Needs Chromium on the CI runner</t>
   </si>
   <si>
-    <t xml:space="preserve">PF-007</t>
+    <t>PF-007</t>
   </si>
   <si>
     <t xml:space="preserve">Cart page with 3 items – Web Vitals</t>
   </si>
   <si>
-    <t xml:space="preserve">https://www.demoblaze.com/cart.html</t>
+    <t>https://www.demoblaze.com/cart.html</t>
   </si>
   <si>
     <t xml:space="preserve">Guest cart seeded with 3 items via API before page load</t>
@@ -461,76 +579,80 @@
 cart_render_time p(75) &lt; 4000 ms</t>
   </si>
   <si>
+    <t xml:space="preserve">TOTAL RESULTS 
+    checks_total.......: 5       0.19741/s
+    checks_succeeded...: 100.00% 5 out of 5
+    checks_failed......: 0.00%   0 out of 5
+    ✓ cart shows 3 rows
+    CUSTOM
+    cart_render_time...............: avg=2.46s    min=2.14s    med=2.27s    max=3.39s    p(90)=2.94s    p(95)=3.17s   
+    HTTP
+    http_req_duration..............: avg=344.59ms min=269.27ms med=306.89ms max=678.15ms p(90)=409.52ms p(95)=563.63ms
+      { expected_response:true }...: avg=344.59ms min=269.27ms med=306.89ms max=678.15ms p(90)=409.52ms p(95)=563.63ms
+    http_req_failed................: 0.00%  0 out of 31
+    http_reqs......................: 31     1.223942/s
+    EXECUTION
+    iteration_duration.............: avg=4.8s     min=4.41s    med=4.55s    max=5.86s    p(90)=5.4s     p(95)=5.63s   
+    iterations.....................: 5      0.19741/s
+    vus............................: 1      min=1        max=1
+    vus_max........................: 1      min=1        max=1
+    NETWORK
+    data_received..................: 19 kB  746 B/s
+    data_sent......................: 9.4 kB 369 B/s
+    BROWSER
+    browser_data_received..........: 11 MB  422 kB/s
+    browser_data_sent..............: 87 kB  3.4 kB/s
+    browser_http_req_duration......: avg=280.24ms min=26.97ms  med=261.38ms max=1.41s    p(90)=613.96ms p(95)=701.81ms
+    browser_http_req_failed........: 0.00%  0 out of 156
+    WEB_VITALS
+    browser_web_vital_cls..........: avg=0.074864 min=0.074864 med=0.074864 max=0.074864 p(90)=0.074864 p(95)=0.074864
+    browser_web_vital_fcp..........: avg=659.2ms  min=480ms    med=700ms    max=756ms    p(90)=743.2ms  p(95)=749.6ms 
+    browser_web_vital_inp..........: avg=2ms      min=0s       med=0s       max=8ms      p(90)=5.6ms    p(95)=6.79ms  
+    browser_web_vital_lcp..........: avg=940ms    min=768ms    med=980ms    max=1.02s    p(90)=1.01s    p(95)=1.02s   
+    browser_web_vital_ttfb.........: avg=341.45ms min=158.09ms med=396.39ms max=413.7ms  p(90)=406.98ms p(95)=410.34ms</t>
+  </si>
+  <si>
     <t xml:space="preserve">cart_render_time = navigation → last row visible</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="6">
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
+      <sz val="11.000000"/>
+      <color indexed="64"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.000000"/>
       <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="14.000000"/>
+      <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="10.000000"/>
       <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF1F3864"/>
+      <b/>
+      <sz val="11.000000"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
+      <b/>
+      <sz val="10.000000"/>
+      <color indexed="65"/>
       <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="11"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -543,7 +665,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F3864"/>
-        <bgColor rgb="FF333333"/>
+        <bgColor indexed="63"/>
       </patternFill>
     </fill>
     <fill>
@@ -566,14 +688,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFBFBFBF"/>
       </left>
@@ -586,264 +708,555 @@
       <bottom style="thin">
         <color rgb="FFBFBFBF"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+  <cellStyleXfs count="6">
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyProtection="1">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="43" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="41" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="15">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="5" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyProtection="0">
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment horizontal="center"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="3" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="4" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf fontId="1" fillId="5" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="top" wrapText="1"/>
+      <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="2" builtinId="6"/>
+    <cellStyle name="Currency" xfId="3" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="4" builtinId="7"/>
+    <cellStyle name="Percent" xfId="5" builtinId="5"/>
   </cellStyles>
-  <dxfs count="10">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="00FFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFDDEBF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFE2EFDA"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFDDEBF7"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFE2EFDA"/>
-      <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFEB9C"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFC7CE"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF1F3864"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF333333"/>
-    </indexedColors>
-  </colors>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Angsana New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Cordia New"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="">
+  <a:themeElements>
+    <a:clrScheme name="">
+      <a:dk1>
+        <a:srgbClr val="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:srgbClr val="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="">
+      <a:majorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface="Arial"/>
+        <a:cs typeface="Arial"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill>
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+        <a:ln w="38100">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst/>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="63000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+        <a:solidFill>
+          <a:srgbClr val="000000"/>
+        </a:solidFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+</a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col customWidth="1" min="1" max="1" style="0" width="24"/>
+    <col customWidth="1" min="2" max="2" style="0" width="46"/>
+    <col customWidth="1" min="3" max="3" style="0" width="40"/>
+    <col customWidth="1" min="4" max="4" style="0" width="18"/>
+    <col customWidth="1" min="5" max="6" style="0" width="12"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="18" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="18">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="14.25">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -851,7 +1264,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" ht="14.25">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
@@ -859,7 +1272,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" ht="14.25">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -867,7 +1280,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" ht="14.25">
       <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
@@ -875,7 +1288,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" ht="14.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
@@ -883,7 +1296,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" ht="14.25">
       <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
@@ -891,12 +1304,12 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" ht="14.25">
       <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" ht="14.25">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -910,80 +1323,80 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" ht="14.25">
       <c r="A12" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Smoke",Performance!$B:$B,"Login")</f>
+      <c r="B12" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Smoke",Performance!$B:$B,"Login")</f>
         <v>1</v>
       </c>
-      <c r="C12" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Smoke",Performance!$B:$B,"Cart")</f>
+      <c r="C12" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Smoke",Performance!$B:$B,"Cart")</f>
         <v>0</v>
       </c>
-      <c r="D12" s="7" t="n">
-        <f aca="false">SUM(B12:C12)</f>
+      <c r="D12" s="7">
+        <f t="shared" ref="D12:D14" si="0">SUM(B12:C12)</f>
         <v>1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" ht="14.25">
       <c r="A13" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Load",Performance!$B:$B,"Login")</f>
+      <c r="B13" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Load",Performance!$B:$B,"Login")</f>
         <v>1</v>
       </c>
-      <c r="C13" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Load",Performance!$B:$B,"Cart")</f>
+      <c r="C13" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Load",Performance!$B:$B,"Cart")</f>
         <v>3</v>
       </c>
-      <c r="D13" s="7" t="n">
-        <f aca="false">SUM(B13:C13)</f>
+      <c r="D13" s="7">
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" ht="14.25">
       <c r="A14" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B14" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Web Vitals",Performance!$B:$B,"Login")</f>
+      <c r="B14" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Web Vitals",Performance!$B:$B,"Login")</f>
         <v>1</v>
       </c>
-      <c r="C14" s="7" t="n">
-        <f aca="false">COUNTIFS(Performance!$D:$D,"Web Vitals",Performance!$B:$B,"Cart")</f>
+      <c r="C14" s="7">
+        <f>COUNTIFS(Performance!$D:$D,"Web Vitals",Performance!$B:$B,"Cart")</f>
         <v>1</v>
       </c>
-      <c r="D14" s="7" t="n">
-        <f aca="false">SUM(B14:C14)</f>
+      <c r="D14" s="7">
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" ht="14.25">
       <c r="A15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="9" t="n">
-        <f aca="false">SUM(B12:B14)</f>
+      <c r="B15" s="9">
+        <f>SUM(B12:B14)</f>
         <v>3</v>
       </c>
-      <c r="C15" s="9" t="n">
-        <f aca="false">SUM(C12:C14)</f>
+      <c r="C15" s="9">
+        <f>SUM(C12:C14)</f>
         <v>4</v>
       </c>
-      <c r="D15" s="9" t="n">
-        <f aca="false">SUM(D12:D14)</f>
+      <c r="D15" s="9">
+        <f>SUM(D12:D14)</f>
         <v>7</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" ht="14.25">
       <c r="A17" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" ht="14.25">
       <c r="A18" s="5" t="s">
         <v>22</v>
       </c>
@@ -1000,34 +1413,34 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <f aca="false">COUNTIF(Performance!$N:$N,"Pass")</f>
-        <v>3</v>
-      </c>
-      <c r="B19" s="7" t="n">
-        <f aca="false">COUNTIF(Performance!$N:$N,"Fail")</f>
+    <row r="19" ht="14.25">
+      <c r="A19" s="7">
+        <f>COUNTIF(Performance!$N:$N,"Pass")</f>
+        <v>6</v>
+      </c>
+      <c r="B19" s="7">
+        <f>COUNTIF(Performance!$N:$N,"Fail")</f>
+        <v>1</v>
+      </c>
+      <c r="C19" s="7">
+        <f>COUNTIF(Performance!$N:$N,"Blocked")</f>
         <v>0</v>
       </c>
-      <c r="C19" s="7" t="n">
-        <f aca="false">COUNTIF(Performance!$N:$N,"Blocked")</f>
+      <c r="D19" s="7">
+        <f>COUNTIF(Performance!$N:$N,"Not Run")</f>
         <v>0</v>
       </c>
-      <c r="D19" s="7" t="n">
-        <f aca="false">COUNTIF(Performance!$N:$N,"Not Run")</f>
-        <v>4</v>
-      </c>
-      <c r="E19" s="10" t="n">
-        <f aca="false">IFERROR(A19/(A19+B19+C19),0)</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="E19" s="10">
+        <f>IFERROR(A19/(A19+B19+C19),0)</f>
+        <v>0.857142857142857</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
       <c r="A21" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" ht="14.25">
       <c r="A22" s="5" t="s">
         <v>28</v>
       </c>
@@ -1041,7 +1454,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" ht="14.25">
       <c r="A23" s="11" t="s">
         <v>32</v>
       </c>
@@ -1055,7 +1468,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" ht="14.25">
       <c r="A24" s="11" t="s">
         <v>36</v>
       </c>
@@ -1069,7 +1482,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" ht="14.25">
       <c r="A25" s="11" t="s">
         <v>40</v>
       </c>
@@ -1084,42 +1497,39 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr filterMode="0">
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:P8"/>
-  <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.63671875" defaultRowHeight="14.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="30.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="31.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="30"/>
+    <col customWidth="1" min="1" max="2" style="0" width="9"/>
+    <col customWidth="1" min="3" max="3" style="0" width="34"/>
+    <col customWidth="1" min="4" max="4" style="0" width="12"/>
+    <col customWidth="1" min="5" max="5" style="0" width="9"/>
+    <col customWidth="1" min="6" max="6" style="0" width="26"/>
+    <col customWidth="1" min="7" max="7" style="0" width="28"/>
+    <col customWidth="1" min="8" max="8" style="0" width="26"/>
+    <col customWidth="1" min="9" max="9" style="0" width="30.989999999999998"/>
+    <col customWidth="1" min="10" max="10" style="0" width="28"/>
+    <col customWidth="1" min="11" max="11" style="0" width="31.5"/>
+    <col customWidth="1" min="12" max="12" style="0" width="11"/>
+    <col customWidth="1" min="13" max="13" style="0" width="36"/>
+    <col customWidth="1" min="14" max="14" style="0" width="11"/>
+    <col customWidth="1" min="15" max="15" style="0" width="28"/>
+    <col customWidth="1" min="16" max="16" style="0" width="30"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="24.6" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" ht="24.600000000000001" customHeight="1">
       <c r="A1" s="5" t="s">
         <v>43</v>
       </c>
@@ -1169,7 +1579,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="73.1" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="2" ht="73.099999999999994" customHeight="1">
       <c r="A2" s="11" t="s">
         <v>58</v>
       </c>
@@ -1219,7 +1629,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="99.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" ht="99.5" customHeight="1">
       <c r="A3" s="11" t="s">
         <v>72</v>
       </c>
@@ -1269,7 +1679,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" ht="90" customHeight="1">
       <c r="A4" s="11" t="s">
         <v>79</v>
       </c>
@@ -1312,41 +1722,43 @@
       <c r="N4" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="O4" s="11"/>
+      <c r="O4" s="11" t="s">
+        <v>86</v>
+      </c>
       <c r="P4" s="11" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="33.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" ht="129.65000000000001" customHeight="1">
       <c r="A5" s="11" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B5" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D5" s="13" t="s">
         <v>19</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>74</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K5" s="11" t="s">
         <v>66</v>
@@ -1358,20 +1770,22 @@
         <v>85</v>
       </c>
       <c r="N5" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="O5" s="11"/>
+        <v>23</v>
+      </c>
+      <c r="O5" s="11" t="s">
+        <v>95</v>
+      </c>
       <c r="P5" s="11"/>
     </row>
-    <row r="6" customFormat="false" ht="56.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" ht="118.3" customHeight="1">
       <c r="A6" s="11" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B6" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D6" s="13" t="s">
         <v>19</v>
@@ -1380,7 +1794,7 @@
         <v>60</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G6" s="11" t="s">
         <v>82</v>
@@ -1389,13 +1803,13 @@
         <v>74</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="J6" s="11" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="K6" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="L6" s="11" t="s">
         <v>67</v>
@@ -1404,135 +1818,232 @@
         <v>85</v>
       </c>
       <c r="N6" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="O6" s="11"/>
+        <v>22</v>
+      </c>
+      <c r="O6" s="11" t="s">
+        <v>102</v>
+      </c>
       <c r="P6" s="11" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="49.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7" ht="91.299999999999997" customHeight="1">
       <c r="A7" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="B7" s="11" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D7" s="14" t="s">
         <v>20</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I7" s="11" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="J7" s="11" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="K7" s="11" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="L7" s="11" t="s">
         <v>67</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="N7" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="O7" s="11"/>
+        <v>22</v>
+      </c>
+      <c r="O7" s="11" t="s">
+        <v>113</v>
+      </c>
       <c r="P7" s="11" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="49.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" ht="109.65000000000001" customHeight="1">
       <c r="A8" s="11" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B8" s="11" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D8" s="14" t="s">
         <v>20</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="G8" s="11" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H8" s="11" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="J8" s="11" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K8" s="11" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="L8" s="11" t="s">
         <v>67</v>
       </c>
       <c r="M8" s="11" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="N8" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="O8" s="11"/>
+        <v>22</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>122</v>
+      </c>
       <c r="P8" s="11" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P8"/>
-  <conditionalFormatting sqref="N2:N8">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
-      <formula>"Pass"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
-      <formula>"Fail"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
-      <formula>"Blocked"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="N2:N8" type="list">
-      <formula1>"Not Run,Pass,Fail,Blocked,Skipped"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <printOptions headings="0" gridLines="0" horizontalCentered="0" verticalCentered="0"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51181102362204689" footer="0.51181102362204689"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
+      <x14:conditionalFormattings>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N2:N8</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N2:N8</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N2:N8</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="2" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Pass"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFC6EFCE"/>
+                  <bgColor rgb="FFC6EFCE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N5</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="3" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Fail"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFC7CE"/>
+                  <bgColor rgb="FFFFC7CE"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N5</xm:sqref>
+        </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="cellIs" priority="4" aboveAverage="0" operator="equal" rank="0" text="">
+            <xm:f>"Blocked"</xm:f>
+            <x14:dxf>
+              <fill>
+                <patternFill patternType="solid">
+                  <fgColor rgb="FFFFEB9C"/>
+                  <bgColor rgb="FFFFEB9C"/>
+                </patternFill>
+              </fill>
+            </x14:dxf>
+          </x14:cfRule>
+          <xm:sqref>N5</xm:sqref>
+        </x14:conditionalFormatting>
+      </x14:conditionalFormattings>
+    </ext>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2" disablePrompts="0">
+        <x14:dataValidation xr:uid="{17A52E6C-F606-49FE-91FE-22B13D4AD23F}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>N2:N4 N6:N8</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation xr:uid="{36891995-F139-430C-A9F3-BB4D647711E1}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="0" showInputMessage="0">
+          <x14:formula1>
+            <xm:f>"Not Run,Pass,Fail,Blocked,Skipped"</xm:f>
+          </x14:formula1>
+          <x14:formula2>
+            <xm:f>0</xm:f>
+          </x14:formula2>
+          <xm:sqref>N5</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>